<commit_message>
Preenche com zeros à esquerda os campos de Ocorrências
</commit_message>
<xml_diff>
--- a/dados/InPut Dot_01 a 310126_AplicaçãoId32_1_a_5.xlsx
+++ b/dados/InPut Dot_01 a 310126_AplicaçãoId32_1_a_5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergio.franco_boxnet\Documents\Git\bradesco-rpa-32\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4C178C-FEE0-43EC-92EB-78D887797422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEE56BB1-CD15-4C84-A8EE-96EBC4362AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6624" yWindow="1128" windowWidth="11928" windowHeight="10368" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33930" yWindow="1980" windowWidth="21555" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MVC32" sheetId="1" r:id="rId1"/>
@@ -126,6 +126,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="00"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -203,13 +206,17 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -520,7 +527,7 @@
   <cols>
     <col min="1" max="4" width="8.88671875" style="2"/>
     <col min="5" max="5" width="20.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.21875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.21875" style="5" customWidth="1"/>
     <col min="7" max="7" width="20.77734375" style="2" customWidth="1"/>
     <col min="8" max="8" width="16.5546875" style="2" customWidth="1"/>
     <col min="9" max="9" width="20.77734375" style="2" customWidth="1"/>
@@ -550,7 +557,7 @@
       <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -597,7 +604,7 @@
       <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="5">
         <v>5</v>
       </c>
     </row>
@@ -648,7 +655,7 @@
       <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="5">
         <v>1</v>
       </c>
     </row>
@@ -665,7 +672,7 @@
       <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="5">
         <v>10</v>
       </c>
     </row>

</xml_diff>